<commit_message>
notas projetos... junho corrigidas, okkk
</commit_message>
<xml_diff>
--- a/05 Others/2026.1 Avaliação Projetos/Turma Python RAD - ARA0095 Turma 3001  PRESENCIAL Wyden UniRuy 2026_1.xlsx
+++ b/05 Others/2026.1 Avaliação Projetos/Turma Python RAD - ARA0095 Turma 3001  PRESENCIAL Wyden UniRuy 2026_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YduqsArea1\Avaliações Yduqs 2022_2 BDQ 2023_1 2024_2\2026.1 Avaliação Projetos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C6D9CC-3101-4B2D-86A0-AECF1ECDD738}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{336010AF-8328-4194-80E0-91699B3F5194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{DD6ED3E7-57DF-4A52-9E4C-63B0F7661B3D}"/>
   </bookViews>
@@ -352,7 +352,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -545,51 +545,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -630,24 +591,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="1" applyBorder="1"/>
@@ -660,6 +609,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -1046,11 +1002,11 @@
       <c r="A2" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="16">
+      <c r="B2" s="8">
         <v>5</v>
       </c>
       <c r="C2" s="8">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D2" s="8">
         <v>0</v>
@@ -1062,17 +1018,17 @@
         <v>0.9</v>
       </c>
       <c r="G2" s="9">
-        <f>$C$2/7*4</f>
-        <v>0</v>
+        <f>C2/8*4</f>
+        <v>3.6</v>
       </c>
       <c r="H2" s="10">
         <v>5</v>
       </c>
       <c r="I2" s="10">
         <f>G2+H2</f>
-        <v>5</v>
-      </c>
-      <c r="J2" s="24" t="s">
+        <v>8.6</v>
+      </c>
+      <c r="J2" s="20" t="s">
         <v>44</v>
       </c>
       <c r="K2" t="s">
@@ -1083,11 +1039,11 @@
       <c r="A3" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="17">
+      <c r="B3" s="4">
         <v>10</v>
       </c>
       <c r="C3" s="4">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="D3" s="4">
         <v>0</v>
@@ -1099,20 +1055,20 @@
         <v>0.3</v>
       </c>
       <c r="G3" s="5">
-        <f t="shared" ref="G3:G21" si="0">$C$2/7*4</f>
-        <v>0</v>
+        <f t="shared" ref="G3:G21" si="0">C3/8*4</f>
+        <v>2.4</v>
       </c>
       <c r="H3" s="6">
         <v>6</v>
       </c>
       <c r="I3" s="6">
         <f t="shared" ref="I3:I21" si="1">G3+H3</f>
-        <v>6</v>
-      </c>
-      <c r="J3" s="23" t="s">
+        <v>8.4</v>
+      </c>
+      <c r="J3" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="25" t="s">
+      <c r="K3" s="21" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1120,11 +1076,11 @@
       <c r="A4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="17">
+      <c r="B4" s="4">
         <v>16</v>
       </c>
       <c r="C4" s="4">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D4" s="4">
         <v>0</v>
@@ -1137,19 +1093,19 @@
       </c>
       <c r="G4" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="H4" s="6">
         <v>6</v>
       </c>
       <c r="I4" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J4" s="23" t="s">
+        <v>9.6</v>
+      </c>
+      <c r="J4" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="K4" s="26" t="s">
+      <c r="K4" s="22" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1157,11 +1113,11 @@
       <c r="A5" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="17">
+      <c r="B5" s="4">
         <v>7</v>
       </c>
       <c r="C5" s="4">
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="D5" s="4">
         <v>0</v>
@@ -1174,19 +1130,19 @@
       </c>
       <c r="G5" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="H5" s="6">
         <v>6</v>
       </c>
       <c r="I5" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J5" s="23" t="s">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="J5" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="K5" s="25" t="s">
+      <c r="K5" s="21" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1194,11 +1150,11 @@
       <c r="A6" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="4">
         <v>9</v>
       </c>
       <c r="C6" s="4">
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="D6" s="4">
         <v>0</v>
@@ -1211,19 +1167,19 @@
       </c>
       <c r="G6" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="H6" s="6">
         <v>6</v>
       </c>
       <c r="I6" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J6" s="23" t="s">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="J6" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="K6" s="25" t="s">
+      <c r="K6" s="21" t="s">
         <v>51</v>
       </c>
     </row>
@@ -1231,11 +1187,11 @@
       <c r="A7" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="4">
         <v>14</v>
       </c>
       <c r="C7" s="4">
-        <v>0</v>
+        <v>6.4</v>
       </c>
       <c r="D7" s="4">
         <v>0</v>
@@ -1248,31 +1204,31 @@
       </c>
       <c r="G7" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H7" s="6">
         <v>6</v>
       </c>
       <c r="I7" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J7" s="23" t="s">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="J7" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="K7" s="25" t="s">
+      <c r="K7" s="21" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="17">
+      <c r="B8" s="4">
         <v>17</v>
       </c>
       <c r="C8" s="4">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D8" s="4">
         <v>0</v>
@@ -1285,31 +1241,31 @@
       </c>
       <c r="G8" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="H8" s="6">
         <v>2.5</v>
       </c>
       <c r="I8" s="6">
         <f t="shared" si="1"/>
-        <v>2.5</v>
-      </c>
-      <c r="J8" s="23" t="s">
+        <v>6.1</v>
+      </c>
+      <c r="J8" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="K8" s="27" t="s">
+      <c r="K8" s="23" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="4">
         <v>17</v>
       </c>
       <c r="C9" s="4">
-        <v>0</v>
+        <v>6.4</v>
       </c>
       <c r="D9" s="4">
         <v>0</v>
@@ -1322,19 +1278,19 @@
       </c>
       <c r="G9" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="H9" s="6">
         <v>2.5</v>
       </c>
       <c r="I9" s="6">
         <f t="shared" si="1"/>
-        <v>2.5</v>
-      </c>
-      <c r="J9" s="23" t="s">
+        <v>5.7</v>
+      </c>
+      <c r="J9" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="27" t="s">
+      <c r="K9" s="23" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1342,11 +1298,11 @@
       <c r="A10" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="4">
         <v>1</v>
       </c>
       <c r="C10" s="4">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D10" s="4">
         <v>0</v>
@@ -1359,19 +1315,19 @@
       </c>
       <c r="G10" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="H10" s="6">
         <v>6</v>
       </c>
       <c r="I10" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J10" s="23" t="s">
+        <v>9.6</v>
+      </c>
+      <c r="J10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="K10" s="25" t="s">
+      <c r="K10" s="21" t="s">
         <v>53</v>
       </c>
     </row>
@@ -1379,11 +1335,11 @@
       <c r="A11" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="4">
         <v>3</v>
       </c>
       <c r="C11" s="4">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D11" s="4">
         <v>0</v>
@@ -1396,19 +1352,19 @@
       </c>
       <c r="G11" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="H11" s="6">
         <v>6</v>
       </c>
       <c r="I11" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J11" s="23" t="s">
+        <v>9.6</v>
+      </c>
+      <c r="J11" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="K11" s="25" t="s">
+      <c r="K11" s="21" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1416,11 +1372,11 @@
       <c r="A12" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="17">
+      <c r="B12" s="4">
         <v>4</v>
       </c>
       <c r="C12" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D12" s="4">
         <v>0</v>
@@ -1433,19 +1389,19 @@
       </c>
       <c r="G12" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H12" s="6">
         <v>6</v>
       </c>
       <c r="I12" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J12" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="J12" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="K12" s="28" t="s">
+      <c r="K12" s="24" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1453,11 +1409,11 @@
       <c r="A13" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B13" s="17">
+      <c r="B13" s="4">
         <v>6</v>
       </c>
       <c r="C13" s="4">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D13" s="4">
         <v>0</v>
@@ -1470,16 +1426,16 @@
       </c>
       <c r="G13" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="H13" s="6">
         <v>4</v>
       </c>
       <c r="I13" s="6">
         <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="J13" s="23" t="s">
+        <v>7.6</v>
+      </c>
+      <c r="J13" s="19" t="s">
         <v>56</v>
       </c>
       <c r="K13" t="s">
@@ -1490,11 +1446,11 @@
       <c r="A14" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="17">
+      <c r="B14" s="4">
         <v>2</v>
       </c>
       <c r="C14" s="4">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="D14" s="4">
         <v>0</v>
@@ -1507,19 +1463,19 @@
       </c>
       <c r="G14" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="H14" s="6">
         <v>6</v>
       </c>
       <c r="I14" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J14" s="23" t="s">
+        <v>8.4</v>
+      </c>
+      <c r="J14" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="K14" s="25" t="s">
+      <c r="K14" s="21" t="s">
         <v>57</v>
       </c>
     </row>
@@ -1527,11 +1483,11 @@
       <c r="A15" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="17">
+      <c r="B15" s="4">
         <v>12</v>
       </c>
       <c r="C15" s="4">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D15" s="4">
         <v>0</v>
@@ -1544,19 +1500,19 @@
       </c>
       <c r="G15" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H15" s="6">
         <v>6</v>
       </c>
       <c r="I15" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J15" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="J15" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="K15" s="25" t="s">
+      <c r="K15" s="21" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1564,11 +1520,11 @@
       <c r="A16" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="17">
+      <c r="B16" s="4">
         <v>11</v>
       </c>
       <c r="C16" s="4">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D16" s="4">
         <v>0</v>
@@ -1581,29 +1537,29 @@
       </c>
       <c r="G16" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="H16" s="6">
         <v>6</v>
       </c>
       <c r="I16" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J16" s="23" t="s">
+        <v>9.6</v>
+      </c>
+      <c r="J16" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="K16" s="25" t="s">
+      <c r="K16" s="21" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="22"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="4">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D17" s="4">
         <v>0</v>
@@ -1616,29 +1572,29 @@
       </c>
       <c r="G17" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H17" s="6">
-        <v>0</v>
-      </c>
-      <c r="I17" s="6">
+        <v>3.6</v>
+      </c>
+      <c r="H17" s="28">
+        <v>0</v>
+      </c>
+      <c r="I17" s="28">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J17" s="19" t="s">
+        <v>3.6</v>
+      </c>
+      <c r="J17" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="K17" s="27"/>
+      <c r="K17" s="23"/>
     </row>
     <row r="18" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="17">
+      <c r="B18" s="4">
         <v>13</v>
       </c>
       <c r="C18" s="4">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="D18" s="4">
         <v>0</v>
@@ -1651,16 +1607,16 @@
       </c>
       <c r="G18" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="H18" s="6">
         <v>6</v>
       </c>
       <c r="I18" s="6">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-      <c r="J18" s="23" t="s">
+        <v>7.6</v>
+      </c>
+      <c r="J18" s="19" t="s">
         <v>43</v>
       </c>
       <c r="K18" t="s">
@@ -1671,11 +1627,11 @@
       <c r="A19" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="17">
+      <c r="B19" s="4">
         <v>5</v>
       </c>
       <c r="C19" s="4">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D19" s="4">
         <v>0</v>
@@ -1688,16 +1644,16 @@
       </c>
       <c r="G19" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="H19" s="6">
         <v>5</v>
       </c>
       <c r="I19" s="6">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="J19" s="23" t="s">
+        <v>8.6</v>
+      </c>
+      <c r="J19" s="19" t="s">
         <v>44</v>
       </c>
       <c r="K19" t="s">
@@ -1708,11 +1664,11 @@
       <c r="A20" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="17">
+      <c r="B20" s="4">
         <v>15</v>
       </c>
       <c r="C20" s="4">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D20" s="4">
         <v>0</v>
@@ -1725,27 +1681,27 @@
       </c>
       <c r="G20" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="H20" s="6">
         <v>4.3</v>
       </c>
       <c r="I20" s="6">
         <f t="shared" si="1"/>
-        <v>4.3</v>
-      </c>
-      <c r="J20" s="23" t="s">
+        <v>7.9</v>
+      </c>
+      <c r="J20" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="26" t="s">
+      <c r="K20" s="22" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="20" t="s">
+      <c r="A21" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="B21" s="21"/>
+      <c r="B21" s="27"/>
       <c r="C21" s="12">
         <v>0</v>
       </c>
@@ -1769,10 +1725,10 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J21" s="29" t="s">
+      <c r="J21" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="K21" s="27"/>
+      <c r="K21" s="23"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">

</xml_diff>